<commit_message>
new GUI #5 03042026 update, single person app GUI
</commit_message>
<xml_diff>
--- a/excel/בועז_בילגורי_תוצאות_ריצה.xlsx
+++ b/excel/בועז_בילגורי_תוצאות_ריצה.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P62"/>
+  <dimension ref="A1:P63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -971,7 +971,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>09/01/2026</t>
+          <t>27/02/2026</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -986,250 +986,254 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Tiberias Marathon 2026</t>
+          <t>מרתון תל אביב 2026</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2582</t>
+          <t>526</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>01:40:47</t>
+          <t>03:06:27</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>01:40:02</t>
+          <t>03:06:19</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>21000</t>
+          <t>42195</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>456</t>
+          <t>124</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>416</t>
+          <t>115</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>71</t>
+          <t>14</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>M45-49</t>
-        </is>
-      </c>
-      <c r="M10" t="inlineStr"/>
+          <t>M45-49 Marathon</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>1981</t>
+        </is>
+      </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>21K</t>
+          <t>42K</t>
         </is>
       </c>
       <c r="O10" s="2" t="n">
-        <v>0.06946759259259259</v>
+        <v>0.1293865740740741</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>19/12/2025</t>
+          <t>09/01/2026</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>בילגורי</t>
+          <t>בועז</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>בועז</t>
+          <t>בילגורי</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>מרוץ המכבים 2025</t>
+          <t>Tiberias Marathon 2026</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>48</t>
+          <t>2582</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>00:40:27</t>
+          <t>01:40:47</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>00:40:25</t>
+          <t>01:40:02</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>10 ק"מ</t>
+          <t>21000</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>456</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>416</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>71</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>40-49 M</t>
+          <t>M45-49</t>
         </is>
       </c>
       <c r="M11" t="inlineStr"/>
       <c r="N11" t="inlineStr">
         <is>
-          <t>10K</t>
+          <t>21K</t>
         </is>
       </c>
       <c r="O11" s="2" t="n">
-        <v>0.02806712962962963</v>
+        <v>0.06946759259259259</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>05/12/2025</t>
+          <t>19/12/2025</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>בועז</t>
+          <t>בילגורי</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>בילגורי</t>
+          <t>בועז</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>מרוץ חבר 2025</t>
+          <t>מרוץ המכבים 2025</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1239</t>
+          <t>48</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>00:58:10</t>
+          <t>00:40:27</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>00:00:00</t>
+          <t>00:40:25</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>15000</t>
+          <t>10 ק"מ</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>4</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>גברים 40-49, 15 ק"מ</t>
+          <t>40-49 M</t>
         </is>
       </c>
       <c r="M12" t="inlineStr"/>
       <c r="N12" t="inlineStr">
         <is>
-          <t>15K</t>
+          <t>10K</t>
         </is>
       </c>
       <c r="O12" s="2" t="n">
-        <v>0.04039351851851852</v>
+        <v>0.02806712962962963</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>21/11/2025</t>
+          <t>05/12/2025</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>בילגורי</t>
+          <t>בועז</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>בועז</t>
+          <t>בילגורי</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>מרוץ באר יעקב 2025</t>
+          <t>מרוץ חבר 2025</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>5047</t>
+          <t>1239</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>00:18:32</t>
+          <t>00:58:10</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>00:18:31</t>
+          <t>00:00:00</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>5000</t>
+          <t>15000</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>6</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
@@ -1239,124 +1243,124 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>40-49 M</t>
+          <t>גברים 40-49, 15 ק"מ</t>
         </is>
       </c>
       <c r="M13" t="inlineStr"/>
       <c r="N13" t="inlineStr">
         <is>
-          <t>5K</t>
+          <t>15K</t>
         </is>
       </c>
       <c r="O13" s="2" t="n">
-        <v>0.0128587962962963</v>
+        <v>0.04039351851851852</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>20/11/2025</t>
+          <t>21/11/2025</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>בועז</t>
+          <t>בילגורי</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>בילגורי</t>
+          <t>בועז</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>מרוץ הלילה של פתח תקווה 2025</t>
+          <t>מרוץ באר יעקב 2025</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>10105</t>
+          <t>5047</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>00:37:44</t>
+          <t>00:18:32</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>00:00:00</t>
+          <t>00:18:31</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>10 ק"מ</t>
+          <t>5000</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>3</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>2</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>גברים 20-49 ,10 ק"מ</t>
+          <t>40-49 M</t>
         </is>
       </c>
       <c r="M14" t="inlineStr"/>
       <c r="N14" t="inlineStr">
         <is>
-          <t>10K</t>
+          <t>5K</t>
         </is>
       </c>
       <c r="O14" s="2" t="n">
-        <v>0.0262037037037037</v>
+        <v>0.0128587962962963</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>07/11/2025</t>
+          <t>20/11/2025</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>בילגורי</t>
+          <t>בועז</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>בועז</t>
+          <t>בילגורי</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>מרוץ לוד 2025</t>
+          <t>מרוץ הלילה של פתח תקווה 2025</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>1159</t>
+          <t>10105</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>00:38:13</t>
+          <t>00:37:44</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>00:38:12</t>
+          <t>00:00:00</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1366,22 +1370,22 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>11</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>11</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>9</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>40-49 M</t>
+          <t>גברים 20-49 ,10 ק"מ</t>
         </is>
       </c>
       <c r="M15" t="inlineStr"/>
@@ -1391,84 +1395,84 @@
         </is>
       </c>
       <c r="O15" s="2" t="n">
-        <v>0.02652777777777778</v>
+        <v>0.0262037037037037</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>29/10/2025</t>
+          <t>07/11/2025</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>בועז</t>
+          <t>בילגורי</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>בילגורי</t>
+          <t>בועז</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>מרוץ הלילה של תל 2025</t>
+          <t>מרוץ לוד 2025</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>1407</t>
+          <t>1159</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>00:59:51</t>
+          <t>00:38:13</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>00:00:00</t>
+          <t>00:38:12</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>15000</t>
+          <t>10 ק"מ</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>18</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>16</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>גברים 40-49, 15 ק"מ</t>
+          <t>40-49 M</t>
         </is>
       </c>
       <c r="M16" t="inlineStr"/>
       <c r="N16" t="inlineStr">
         <is>
-          <t>15K</t>
+          <t>10K</t>
         </is>
       </c>
       <c r="O16" s="2" t="n">
-        <v>0.0415625</v>
+        <v>0.02652777777777778</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>10/10/2025</t>
+          <t>29/10/2025</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1483,55 +1487,63 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>מרוץ נחל שורק 2025</t>
+          <t>מרוץ הלילה של תל 2025</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>43</t>
+          <t>1407</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>00:36:44</t>
+          <t>00:59:51</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>00:36:42</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr"/>
+          <t>00:00:00</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>15000</t>
+        </is>
+      </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>ותיקים 40-49</t>
+          <t>גברים 40-49, 15 ק"מ</t>
         </is>
       </c>
       <c r="M17" t="inlineStr"/>
-      <c r="N17" t="inlineStr"/>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>15K</t>
+        </is>
+      </c>
       <c r="O17" s="2" t="n">
-        <v>0.02548611111111111</v>
+        <v>0.0415625</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>12/06/2025</t>
+          <t>10/10/2025</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1546,42 +1558,38 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>מרוץ הלילה של מודיעין 2025</t>
+          <t>מרוץ נחל שורק 2025</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>67</t>
+          <t>43</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>00:19:18</t>
+          <t>00:36:44</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>00:19:17</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>5000</t>
-        </is>
-      </c>
+          <t>00:36:42</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>13</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>13</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
@@ -1590,19 +1598,15 @@
         </is>
       </c>
       <c r="M18" t="inlineStr"/>
-      <c r="N18" t="inlineStr">
-        <is>
-          <t>5K</t>
-        </is>
-      </c>
+      <c r="N18" t="inlineStr"/>
       <c r="O18" s="2" t="n">
-        <v>0.0133912037037037</v>
+        <v>0.02548611111111111</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>28/04/2025</t>
+          <t>12/06/2025</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1617,201 +1621,201 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>מרוץ הלילה בחורשת הבנים 2025</t>
+          <t>מרוץ הלילה של מודיעין 2025</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>2876</t>
+          <t>67</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>00:27:42</t>
+          <t>00:19:18</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>00:27:41</t>
+          <t>00:19:17</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>7000</t>
+          <t>5000</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
           <t>1</t>
         </is>
       </c>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="K19" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>כללי גברים</t>
+          <t>ותיקים 40-49</t>
         </is>
       </c>
       <c r="M19" t="inlineStr"/>
-      <c r="N19" t="inlineStr"/>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>5K</t>
+        </is>
+      </c>
       <c r="O19" s="2" t="n">
-        <v>0.01922453703703704</v>
+        <v>0.0133912037037037</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>25/04/2025</t>
+          <t>28/04/2025</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>בילגורי</t>
+          <t>בועז</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>בועז</t>
+          <t>בילגורי</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>מרוץ שפיר 2025</t>
+          <t>מרוץ הלילה בחורשת הבנים 2025</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>1019</t>
+          <t>2876</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>00:38:48</t>
+          <t>00:27:42</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>00:38:47</t>
+          <t>00:27:41</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>10 ק"מ</t>
+          <t>7000</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>1</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>40-49 M</t>
+          <t>כללי גברים</t>
         </is>
       </c>
       <c r="M20" t="inlineStr"/>
-      <c r="N20" t="inlineStr">
-        <is>
-          <t>10K</t>
-        </is>
-      </c>
+      <c r="N20" t="inlineStr"/>
       <c r="O20" s="2" t="n">
-        <v>0.02693287037037037</v>
+        <v>0.01922453703703704</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>04/04/2025</t>
+          <t>25/04/2025</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>בועז</t>
+          <t>בילגורי</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>בילגורי</t>
+          <t>בועז</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Jerusalem Marathon 2025</t>
+          <t>מרוץ שפיר 2025</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>23435</t>
+          <t>1019</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>01:26:24</t>
+          <t>00:38:48</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>00:00:00</t>
+          <t>00:38:47</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>21000</t>
+          <t>10 ק"מ</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>35</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>6</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>M40-44, 21K</t>
+          <t>40-49 M</t>
         </is>
       </c>
       <c r="M21" t="inlineStr"/>
       <c r="N21" t="inlineStr">
         <is>
-          <t>21K</t>
+          <t>10K</t>
         </is>
       </c>
       <c r="O21" s="2" t="n">
-        <v>0.06</v>
+        <v>0.02693287037037037</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>28/03/2025</t>
+          <t>04/04/2025</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1826,104 +1830,108 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>מרוץ מודיעין 2025</t>
+          <t>Jerusalem Marathon 2025</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>105</t>
+          <t>23435</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>00:39:40</t>
+          <t>01:26:24</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>00:39:35</t>
+          <t>00:00:00</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>10 ק"מ</t>
+          <t>21000</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>35</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>32</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>ותיקים 40-49</t>
+          <t>M40-44, 21K</t>
         </is>
       </c>
       <c r="M22" t="inlineStr"/>
       <c r="N22" t="inlineStr">
         <is>
-          <t>10K</t>
+          <t>21K</t>
         </is>
       </c>
       <c r="O22" s="2" t="n">
-        <v>0.02748842592592593</v>
+        <v>0.06</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>07/03/2025</t>
+          <t>28/03/2025</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>בילגורי</t>
+          <t>בועז</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>בועז</t>
+          <t>בילגורי</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>מרוץ נס ציונה 2025</t>
+          <t>מרוץ מודיעין 2025</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>5176</t>
+          <t>105</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>00:17:59</t>
+          <t>00:39:40</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>00:17:59</t>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr"/>
+          <t>00:39:35</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>10 ק"מ</t>
+        </is>
+      </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
@@ -1933,90 +1941,86 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>40-49 M</t>
+          <t>ותיקים 40-49</t>
         </is>
       </c>
       <c r="M23" t="inlineStr"/>
-      <c r="N23" t="inlineStr"/>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>10K</t>
+        </is>
+      </c>
       <c r="O23" s="2" t="n">
-        <v>0.01248842592592593</v>
+        <v>0.02748842592592593</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>03/01/2025</t>
+          <t>07/03/2025</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>בועז</t>
+          <t>בילגורי</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>בילגורי</t>
+          <t>בועז</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Tiberias Marathon 2025</t>
+          <t>מרוץ נס ציונה 2025</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>405</t>
+          <t>5176</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>02:57:21</t>
+          <t>00:17:59</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>02:57:17</t>
-        </is>
-      </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>42195</t>
-        </is>
-      </c>
+          <t>00:17:59</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr"/>
       <c r="I24" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>5</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>5</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>M 40-44 ,Marathon</t>
+          <t>40-49 M</t>
         </is>
       </c>
       <c r="M24" t="inlineStr"/>
-      <c r="N24" t="inlineStr">
-        <is>
-          <t>42K</t>
-        </is>
-      </c>
+      <c r="N24" t="inlineStr"/>
       <c r="O24" s="2" t="n">
-        <v>0.1231134259259259</v>
+        <v>0.01248842592592593</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>12/12/2024</t>
+          <t>03/01/2025</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -2031,63 +2035,63 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>מרוץ בית שמש 2024</t>
+          <t>Tiberias Marathon 2025</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>620</t>
+          <t>405</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>00:38:39</t>
+          <t>02:57:21</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>00:38:37</t>
+          <t>02:57:17</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>10 ק"מ</t>
+          <t>42195</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>21</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>20</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>ותיקים 40-59</t>
+          <t>M 40-44 ,Marathon</t>
         </is>
       </c>
       <c r="M25" t="inlineStr"/>
       <c r="N25" t="inlineStr">
         <is>
-          <t>10K</t>
+          <t>42K</t>
         </is>
       </c>
       <c r="O25" s="2" t="n">
-        <v>0.02681712962962963</v>
+        <v>0.1231134259259259</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>29/11/2024</t>
+          <t>12/12/2024</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -2102,22 +2106,22 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>מרוץ ברנר 2024</t>
+          <t>מרוץ בית שמש 2024</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>1833</t>
+          <t>620</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>00:39:05</t>
+          <t>00:38:39</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>00:39:03</t>
+          <t>00:38:37</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -2127,22 +2131,22 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>ותיקים 40-49</t>
+          <t>ותיקים 40-59</t>
         </is>
       </c>
       <c r="M26" t="inlineStr"/>
@@ -2152,43 +2156,43 @@
         </is>
       </c>
       <c r="O26" s="2" t="n">
-        <v>0.02711805555555555</v>
+        <v>0.02681712962962963</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>22/11/2024</t>
+          <t>29/11/2024</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>בילגורי</t>
+          <t>בועז</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>בועז</t>
+          <t>בילגורי</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>מרוץ באר יעקב 2024</t>
+          <t>מרוץ ברנר 2024</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>1001</t>
+          <t>1833</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>00:37:54</t>
+          <t>00:39:05</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>00:37:54</t>
+          <t>00:39:03</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -2198,22 +2202,22 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>40-49 M</t>
+          <t>ותיקים 40-49</t>
         </is>
       </c>
       <c r="M27" t="inlineStr"/>
@@ -2223,13 +2227,13 @@
         </is>
       </c>
       <c r="O27" s="2" t="n">
-        <v>0.02631944444444444</v>
+        <v>0.02711805555555555</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>01/11/2024</t>
+          <t>22/11/2024</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -2244,27 +2248,27 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>מרוץ מזכרת בתיה 2024</t>
+          <t>מרוץ באר יעקב 2024</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>1013</t>
+          <t>1001</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>00:38:51</t>
+          <t>00:37:54</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>00:38:51</t>
+          <t>00:37:54</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>9800</t>
+          <t>10 ק"מ</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -2279,7 +2283,7 @@
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
@@ -2294,13 +2298,13 @@
         </is>
       </c>
       <c r="O28" s="2" t="n">
-        <v>0.02697916666666667</v>
+        <v>0.02631944444444444</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>12/09/2024</t>
+          <t>01/11/2024</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -2315,42 +2319,42 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>מרוץ הלילה של מודיעין 2024</t>
+          <t>מרוץ מזכרת בתיה 2024</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>3072</t>
+          <t>1013</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>00:19:33</t>
+          <t>00:38:51</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>00:19:32</t>
+          <t>00:38:51</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>5000</t>
+          <t>9800</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
@@ -2361,88 +2365,88 @@
       <c r="M29" t="inlineStr"/>
       <c r="N29" t="inlineStr">
         <is>
-          <t>5K</t>
+          <t>10K</t>
         </is>
       </c>
       <c r="O29" s="2" t="n">
-        <v>0.01356481481481481</v>
+        <v>0.02697916666666667</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>06/06/2024</t>
+          <t>12/09/2024</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>בועז</t>
+          <t>בילגורי</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>בילגורי</t>
+          <t>בועז</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>מרוץ הלילה של פתח תקווה 2024</t>
+          <t>מרוץ הלילה של מודיעין 2024</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>10239</t>
+          <t>3072</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>00:39:09</t>
+          <t>00:19:33</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>00:00:00</t>
+          <t>00:19:32</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>10 ק"מ</t>
+          <t>5000</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>4</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>1</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>גברים 20-49 ,10 ק"מ</t>
+          <t>40-49 M</t>
         </is>
       </c>
       <c r="M30" t="inlineStr"/>
       <c r="N30" t="inlineStr">
         <is>
-          <t>10K</t>
+          <t>5K</t>
         </is>
       </c>
       <c r="O30" s="2" t="n">
-        <v>0.0271875</v>
+        <v>0.01356481481481481</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>09/05/2024</t>
+          <t>06/06/2024</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -2457,59 +2461,63 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>מרוץ הלילה בחורשת הבנים 2024</t>
+          <t>מרוץ הלילה של פתח תקווה 2024</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>892</t>
+          <t>10239</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>00:27:33</t>
+          <t>00:39:09</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>00:27:32</t>
+          <t>00:00:00</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>7000</t>
+          <t>10 ק"מ</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>42</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>41</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>34</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>כללי גברים</t>
+          <t>גברים 20-49 ,10 ק"מ</t>
         </is>
       </c>
       <c r="M31" t="inlineStr"/>
-      <c r="N31" t="inlineStr"/>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>10K</t>
+        </is>
+      </c>
       <c r="O31" s="2" t="n">
-        <v>0.01912037037037037</v>
+        <v>0.0271875</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>17/04/2024</t>
+          <t>09/05/2024</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -2524,93 +2532,89 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>מרוץ הלילה של תל 2024</t>
+          <t>מרוץ הלילה בחורשת הבנים 2024</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>10532</t>
+          <t>892</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>00:43:47</t>
+          <t>00:27:33</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>00:00:00</t>
+          <t>00:27:32</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>10 ק"מ</t>
+          <t>7000</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>302</t>
+          <t>2</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>286</t>
+          <t>2</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>80</t>
+          <t>2</t>
         </is>
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>גברים 40-49, 10 ק"מ</t>
+          <t>כללי גברים</t>
         </is>
       </c>
       <c r="M32" t="inlineStr"/>
-      <c r="N32" t="inlineStr">
-        <is>
-          <t>10K</t>
-        </is>
-      </c>
+      <c r="N32" t="inlineStr"/>
       <c r="O32" s="2" t="n">
-        <v>0.03040509259259259</v>
+        <v>0.01912037037037037</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>12/04/2024</t>
+          <t>17/04/2024</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>בילגורי</t>
+          <t>בועז</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>בועז</t>
+          <t>בילגורי</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>מרוץ נס ציונה 2024</t>
+          <t>מרוץ הלילה של תל 2024</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>1166</t>
+          <t>10532</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>00:38:46</t>
+          <t>00:43:47</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>00:38:44</t>
+          <t>00:00:00</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -2620,22 +2624,22 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>302</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>286</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>80</t>
         </is>
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>40-49 M</t>
+          <t>גברים 40-49, 10 ק"מ</t>
         </is>
       </c>
       <c r="M33" t="inlineStr"/>
@@ -2645,13 +2649,13 @@
         </is>
       </c>
       <c r="O33" s="2" t="n">
-        <v>0.02689814814814815</v>
+        <v>0.03040509259259259</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>05/04/2024</t>
+          <t>12/04/2024</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -2666,22 +2670,22 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>מרוץ מודיעין 2024</t>
+          <t>מרוץ נס ציונה 2024</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>167</t>
+          <t>1166</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>00:38:34</t>
+          <t>00:38:46</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>00:38:33</t>
+          <t>00:38:44</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
@@ -2691,17 +2695,17 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>6</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>3</t>
         </is>
       </c>
       <c r="L34" t="inlineStr">
@@ -2716,13 +2720,13 @@
         </is>
       </c>
       <c r="O34" s="2" t="n">
-        <v>0.02677083333333333</v>
+        <v>0.02689814814814815</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>15/03/2024</t>
+          <t>05/04/2024</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -2737,268 +2741,268 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>מרוץ סביון 2024</t>
+          <t>מרוץ מודיעין 2024</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>338</t>
+          <t>167</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>00:34:52</t>
+          <t>00:38:34</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>00:34:51</t>
-        </is>
-      </c>
-      <c r="H35" t="inlineStr"/>
+          <t>00:38:33</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>10 ק"מ</t>
+        </is>
+      </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>14</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>13</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>40-44M</t>
+          <t>40-49 M</t>
         </is>
       </c>
       <c r="M35" t="inlineStr"/>
-      <c r="N35" t="inlineStr"/>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>10K</t>
+        </is>
+      </c>
       <c r="O35" s="2" t="n">
-        <v>0.02420138888888889</v>
+        <v>0.02677083333333333</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>08/03/2024</t>
+          <t>15/03/2024</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>בועז</t>
+          <t>בילגורי</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>בילגורי</t>
+          <t>בועז</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Jerusalem Marathon 2024</t>
+          <t>מרוץ סביון 2024</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>4735</t>
+          <t>338</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>03:20:27</t>
+          <t>00:34:52</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>03:19:45</t>
-        </is>
-      </c>
-      <c r="H36" t="inlineStr">
-        <is>
-          <t>42195</t>
-        </is>
-      </c>
+          <t>00:34:51</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr"/>
       <c r="I36" t="inlineStr">
         <is>
-          <t>43</t>
+          <t>22</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>21</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>5</t>
         </is>
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>M40-44, 42K</t>
+          <t>40-44M</t>
         </is>
       </c>
       <c r="M36" t="inlineStr"/>
-      <c r="N36" t="inlineStr">
-        <is>
-          <t>42K</t>
-        </is>
-      </c>
+      <c r="N36" t="inlineStr"/>
       <c r="O36" s="2" t="n">
-        <v>0.1387152777777778</v>
+        <v>0.02420138888888889</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>24/02/2024</t>
+          <t>08/03/2024</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>בילגורי</t>
+          <t>בועז</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>בועז</t>
+          <t>בילגורי</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>מרוץ רחובות 2024</t>
+          <t>Jerusalem Marathon 2024</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>1052</t>
+          <t>4735</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>00:48:05</t>
+          <t>03:20:27</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>00:48:05</t>
+          <t>03:19:45</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>10 ק"מ</t>
+          <t>42195</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>43</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>41</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>8</t>
         </is>
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>40-49 M</t>
+          <t>M40-44, 42K</t>
         </is>
       </c>
       <c r="M37" t="inlineStr"/>
       <c r="N37" t="inlineStr">
         <is>
-          <t>10K</t>
+          <t>42K</t>
         </is>
       </c>
       <c r="O37" s="2" t="n">
-        <v>0.0333912037037037</v>
+        <v>0.1387152777777778</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>02/02/2024</t>
+          <t>24/02/2024</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>בועז</t>
+          <t>בילגורי</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>בילגורי</t>
+          <t>בועז</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Dead Sea Marathon 2024</t>
+          <t>מרוץ רחובות 2024</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>350</t>
+          <t>1052</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>03:42:15</t>
+          <t>00:48:05</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>03:39:08</t>
+          <t>00:48:05</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>42195</t>
+          <t>10 ק"מ</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>108</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>95</t>
+          <t>6</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>2</t>
         </is>
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>M 42k40-49</t>
+          <t>40-49 M</t>
         </is>
       </c>
       <c r="M38" t="inlineStr"/>
       <c r="N38" t="inlineStr">
         <is>
-          <t>42K</t>
+          <t>10K</t>
         </is>
       </c>
       <c r="O38" s="2" t="n">
-        <v>0.1521759259259259</v>
+        <v>0.0333912037037037</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>22/09/2023</t>
+          <t>02/02/2024</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -3013,63 +3017,63 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>מרוץ ברנר 2023</t>
+          <t>Dead Sea Marathon 2024</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>520</t>
+          <t>350</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>00:40:43</t>
+          <t>03:42:15</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>00:40:43</t>
+          <t>03:39:08</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>10 ק"מ</t>
+          <t>42195</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>108</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>95</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>42</t>
         </is>
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>ותיקים 40-49</t>
+          <t>M 42k40-49</t>
         </is>
       </c>
       <c r="M39" t="inlineStr"/>
       <c r="N39" t="inlineStr">
         <is>
-          <t>10K</t>
+          <t>42K</t>
         </is>
       </c>
       <c r="O39" s="2" t="n">
-        <v>0.02827546296296296</v>
+        <v>0.1521759259259259</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>15/06/2023</t>
+          <t>22/09/2023</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -3084,37 +3088,37 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>מרוץ הלילה של מודיעין 2023</t>
+          <t>מרוץ ברנר 2023</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>88</t>
+          <t>520</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>00:19:05</t>
+          <t>00:40:43</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>00:00:00</t>
+          <t>00:40:43</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>5000</t>
+          <t>10 ק"מ</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
@@ -3124,23 +3128,23 @@
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>גברים 40-49 ,5 ק"מ</t>
+          <t>ותיקים 40-49</t>
         </is>
       </c>
       <c r="M40" t="inlineStr"/>
       <c r="N40" t="inlineStr">
         <is>
-          <t>5K</t>
+          <t>10K</t>
         </is>
       </c>
       <c r="O40" s="2" t="n">
-        <v>0.01325231481481481</v>
+        <v>0.02827546296296296</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>05/05/2023</t>
+          <t>15/06/2023</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -3155,13 +3159,17 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>מרוץ סביון ה-13 2023</t>
-        </is>
-      </c>
-      <c r="E41" t="inlineStr"/>
+          <t>מרוץ הלילה של מודיעין 2023</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>88</t>
+        </is>
+      </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>00:19:03</t>
+          <t>00:19:05</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -3169,7 +3177,11 @@
           <t>00:00:00</t>
         </is>
       </c>
-      <c r="H41" t="inlineStr"/>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>5000</t>
+        </is>
+      </c>
       <c r="I41" t="inlineStr">
         <is>
           <t>7</t>
@@ -3177,7 +3189,7 @@
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
@@ -3187,161 +3199,153 @@
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>גברים 40-44</t>
+          <t>גברים 40-49 ,5 ק"מ</t>
         </is>
       </c>
       <c r="M41" t="inlineStr"/>
-      <c r="N41" t="inlineStr"/>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>5K</t>
+        </is>
+      </c>
       <c r="O41" s="2" t="n">
-        <v>0.01322916666666667</v>
+        <v>0.01325231481481481</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>24/03/2023</t>
+          <t>05/05/2023</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>בילגורי</t>
+          <t>בועז</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>בועז</t>
+          <t>בילגורי</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>מרוץ נס ציונה 2023</t>
-        </is>
-      </c>
-      <c r="E42" t="inlineStr">
-        <is>
-          <t>1102</t>
-        </is>
-      </c>
+          <t>מרוץ סביון ה-13 2023</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr"/>
       <c r="F42" t="inlineStr">
         <is>
-          <t>00:37:14</t>
+          <t>00:19:03</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>00:37:13</t>
-        </is>
-      </c>
-      <c r="H42" t="inlineStr">
-        <is>
-          <t>10 ק"מ</t>
-        </is>
-      </c>
+          <t>00:00:00</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr"/>
       <c r="I42" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>7</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>8</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>40-49 M</t>
+          <t>גברים 40-44</t>
         </is>
       </c>
       <c r="M42" t="inlineStr"/>
-      <c r="N42" t="inlineStr">
-        <is>
-          <t>10K</t>
-        </is>
-      </c>
+      <c r="N42" t="inlineStr"/>
       <c r="O42" s="2" t="n">
-        <v>0.02584490740740741</v>
+        <v>0.01322916666666667</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>17/03/2023</t>
+          <t>24/03/2023</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>בועז</t>
+          <t>בילגורי</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>בילגורי</t>
+          <t>בועז</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Jerusalem Marathon 2023</t>
+          <t>מרוץ נס ציונה 2023</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>20796</t>
+          <t>1102</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>01:27:51</t>
+          <t>00:37:14</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>00:00:00</t>
+          <t>00:37:13</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>21000</t>
+          <t>10 ק"מ</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>35</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>4</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>M40-44, 21K</t>
+          <t>40-49 M</t>
         </is>
       </c>
       <c r="M43" t="inlineStr"/>
       <c r="N43" t="inlineStr">
         <is>
-          <t>21K</t>
+          <t>10K</t>
         </is>
       </c>
       <c r="O43" s="2" t="n">
-        <v>0.06100694444444445</v>
+        <v>0.02584490740740741</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>03/03/2023</t>
+          <t>17/03/2023</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -3356,63 +3360,63 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>מרוץ ראש העין 2023</t>
+          <t>Jerusalem Marathon 2023</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>772</t>
+          <t>20796</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>00:39:05</t>
+          <t>01:27:51</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>00:39:07</t>
+          <t>00:00:00</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>10 ק"מ</t>
+          <t>21000</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>35</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>32</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>ותיקים 40-49</t>
+          <t>M40-44, 21K</t>
         </is>
       </c>
       <c r="M44" t="inlineStr"/>
       <c r="N44" t="inlineStr">
         <is>
-          <t>10K</t>
+          <t>21K</t>
         </is>
       </c>
       <c r="O44" s="2" t="n">
-        <v>0.02716435185185185</v>
+        <v>0.06100694444444445</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>24/02/2023</t>
+          <t>03/03/2023</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -3427,63 +3431,63 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>מרתון תל אביב 2023</t>
+          <t>מרוץ ראש העין 2023</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>5107</t>
+          <t>772</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>01:26:51</t>
+          <t>00:39:05</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>00:00:00</t>
+          <t>00:39:07</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>21097</t>
+          <t>10 ק"מ</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>197</t>
+          <t>5</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>190</t>
+          <t>5</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
         <is>
-          <t>31</t>
+          <t>2</t>
         </is>
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>גברים 44-40 21K</t>
+          <t>ותיקים 40-49</t>
         </is>
       </c>
       <c r="M45" t="inlineStr"/>
       <c r="N45" t="inlineStr">
         <is>
-          <t>21K</t>
+          <t>10K</t>
         </is>
       </c>
       <c r="O45" s="2" t="n">
-        <v>0.0603125</v>
+        <v>0.02716435185185185</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>17/02/2023</t>
+          <t>24/02/2023</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -3498,17 +3502,17 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>מרוץ דימונה 2023</t>
+          <t>מרתון תל אביב 2023</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>3038</t>
+          <t>5107</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>02:30:09</t>
+          <t>01:26:51</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -3518,39 +3522,43 @@
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>30000</t>
+          <t>21097</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>197</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>190</t>
         </is>
       </c>
       <c r="K46" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>31</t>
         </is>
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>40-49</t>
+          <t>גברים 44-40 21K</t>
         </is>
       </c>
       <c r="M46" t="inlineStr"/>
-      <c r="N46" t="inlineStr"/>
+      <c r="N46" t="inlineStr">
+        <is>
+          <t>21K</t>
+        </is>
+      </c>
       <c r="O46" s="2" t="n">
-        <v>0.1042708333333333</v>
+        <v>0.0603125</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>10/02/2023</t>
+          <t>17/02/2023</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -3565,63 +3573,59 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>מרוץ אור יהודה 2023</t>
+          <t>מרוץ דימונה 2023</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>109</t>
+          <t>3038</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>00:37:47</t>
+          <t>02:30:09</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>00:38:08</t>
+          <t>00:00:00</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>10 ק"מ</t>
+          <t>30000</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>70</t>
+          <t>7</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>68</t>
+          <t>7</t>
         </is>
       </c>
       <c r="K47" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>3</t>
         </is>
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>ותיקים 40-49</t>
+          <t>40-49</t>
         </is>
       </c>
       <c r="M47" t="inlineStr"/>
-      <c r="N47" t="inlineStr">
-        <is>
-          <t>10K</t>
-        </is>
-      </c>
+      <c r="N47" t="inlineStr"/>
       <c r="O47" s="2" t="n">
-        <v>0.02648148148148148</v>
+        <v>0.1042708333333333</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>30/12/2022</t>
+          <t>10/02/2023</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -3636,7 +3640,7 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>מרוץ קרית מלאכי</t>
+          <t>מרוץ אור יהודה 2023</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -3646,12 +3650,12 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>00:39:10</t>
+          <t>00:37:47</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>00:00:00</t>
+          <t>00:38:08</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
@@ -3661,22 +3665,22 @@
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>70</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>68</t>
         </is>
       </c>
       <c r="K48" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>21</t>
         </is>
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>40-49</t>
+          <t>ותיקים 40-49</t>
         </is>
       </c>
       <c r="M48" t="inlineStr"/>
@@ -3686,43 +3690,43 @@
         </is>
       </c>
       <c r="O48" s="2" t="n">
-        <v>0.02719907407407407</v>
+        <v>0.02648148148148148</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>16/12/2022</t>
+          <t>30/12/2022</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>בילגורי</t>
+          <t>בועז</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>בועז</t>
+          <t>בילגורי</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>מרוץ גדרה 2022</t>
+          <t>מרוץ קרית מלאכי</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>1109</t>
+          <t>109</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>00:39:52</t>
+          <t>00:39:10</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>00:39:52</t>
+          <t>00:00:00</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
@@ -3732,12 +3736,12 @@
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>3</t>
         </is>
       </c>
       <c r="K49" t="inlineStr">
@@ -3747,7 +3751,7 @@
       </c>
       <c r="L49" t="inlineStr">
         <is>
-          <t>40-49 M</t>
+          <t>40-49</t>
         </is>
       </c>
       <c r="M49" t="inlineStr"/>
@@ -3757,13 +3761,13 @@
         </is>
       </c>
       <c r="O49" s="2" t="n">
-        <v>0.02768518518518518</v>
+        <v>0.02719907407407407</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>25/11/2022</t>
+          <t>16/12/2022</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -3778,22 +3782,22 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>מרוץ מודיעין 2022</t>
+          <t>מרוץ גדרה 2022</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>1509</t>
+          <t>1109</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>00:38:43</t>
+          <t>00:39:52</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>00:38:43</t>
+          <t>00:39:52</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
@@ -3803,17 +3807,17 @@
       </c>
       <c r="I50" t="inlineStr">
         <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
           <t>2</t>
-        </is>
-      </c>
-      <c r="J50" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="K50" t="inlineStr">
-        <is>
-          <t>1</t>
         </is>
       </c>
       <c r="L50" t="inlineStr">
@@ -3828,13 +3832,13 @@
         </is>
       </c>
       <c r="O50" s="2" t="n">
-        <v>0.02688657407407407</v>
+        <v>0.02768518518518518</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>10/11/2022</t>
+          <t>25/11/2022</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -3849,38 +3853,42 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>מרוץ הלילה של רחובות</t>
+          <t>מרוץ מודיעין 2022</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>1352</t>
+          <t>1509</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>00:34:56</t>
+          <t>00:38:43</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>00:34:53</t>
-        </is>
-      </c>
-      <c r="H51" t="inlineStr"/>
+          <t>00:38:43</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>10 ק"מ</t>
+        </is>
+      </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>2</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>2</t>
         </is>
       </c>
       <c r="K51" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="L51" t="inlineStr">
@@ -3889,183 +3897,179 @@
         </is>
       </c>
       <c r="M51" t="inlineStr"/>
-      <c r="N51" t="inlineStr"/>
+      <c r="N51" t="inlineStr">
+        <is>
+          <t>10K</t>
+        </is>
+      </c>
       <c r="O51" s="2" t="n">
-        <v>0.02422453703703704</v>
+        <v>0.02688657407407407</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>21/10/2022</t>
+          <t>10/11/2022</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>בועז</t>
+          <t>בילגורי</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>בילגורי</t>
+          <t>בועז</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>מרוץ חבר 2022</t>
-        </is>
-      </c>
-      <c r="E52" t="inlineStr"/>
+          <t>מרוץ הלילה של רחובות</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>1352</t>
+        </is>
+      </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>01:01:00</t>
+          <t>00:34:56</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>00:00:00</t>
-        </is>
-      </c>
-      <c r="H52" t="inlineStr">
-        <is>
-          <t>15000</t>
-        </is>
-      </c>
+          <t>00:34:53</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr"/>
       <c r="I52" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>9</t>
         </is>
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>9</t>
         </is>
       </c>
       <c r="K52" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>4</t>
         </is>
       </c>
       <c r="L52" t="inlineStr">
         <is>
-          <t>גברים 30-59, 15 ק"מ</t>
+          <t>40-49 M</t>
         </is>
       </c>
       <c r="M52" t="inlineStr"/>
-      <c r="N52" t="inlineStr">
-        <is>
-          <t>15K</t>
-        </is>
-      </c>
+      <c r="N52" t="inlineStr"/>
       <c r="O52" s="2" t="n">
-        <v>0.04236111111111111</v>
+        <v>0.02422453703703704</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>14/10/2022</t>
+          <t>21/10/2022</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>בילגורי</t>
+          <t>בועז</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>בועז</t>
+          <t>בילגורי</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>מזכרת בתיה 2022</t>
-        </is>
-      </c>
-      <c r="E53" t="inlineStr">
-        <is>
-          <t>74</t>
-        </is>
-      </c>
+          <t>מרוץ חבר 2022</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr"/>
       <c r="F53" t="inlineStr">
         <is>
-          <t>00:38:49</t>
+          <t>01:01:00</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>00:38:49</t>
+          <t>00:00:00</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>10 ק"מ</t>
+          <t>15000</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>17</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>17</t>
         </is>
       </c>
       <c r="K53" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>15</t>
         </is>
       </c>
       <c r="L53" t="inlineStr">
         <is>
-          <t>40-49 M</t>
+          <t>גברים 30-59, 15 ק"מ</t>
         </is>
       </c>
       <c r="M53" t="inlineStr"/>
       <c r="N53" t="inlineStr">
         <is>
-          <t>10K</t>
+          <t>15K</t>
         </is>
       </c>
       <c r="O53" s="2" t="n">
-        <v>0.02695601851851852</v>
+        <v>0.04236111111111111</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>30/09/2022</t>
+          <t>14/10/2022</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>בועז</t>
+          <t>בילגורי</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>בילגורי</t>
+          <t>בועז</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>מרוץ ברנר ה- 6 ע"ש אורלי שחף</t>
+          <t>מזכרת בתיה 2022</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>2889</t>
+          <t>74</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>00:39:37</t>
+          <t>00:38:49</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>00:39:40</t>
+          <t>00:38:49</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
@@ -4075,22 +4079,22 @@
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="K54" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="L54" t="inlineStr">
         <is>
-          <t>ותיקים 40-49</t>
+          <t>40-49 M</t>
         </is>
       </c>
       <c r="M54" t="inlineStr"/>
@@ -4100,13 +4104,13 @@
         </is>
       </c>
       <c r="O54" s="2" t="n">
-        <v>0.0275462962962963</v>
+        <v>0.02695601851851852</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>03/06/2022</t>
+          <t>30/09/2022</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -4121,22 +4125,22 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>מרוץ גני תקווה ה-3</t>
+          <t>מרוץ ברנר ה- 6 ע"ש אורלי שחף</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>546</t>
+          <t>2889</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>00:39:12</t>
+          <t>00:39:37</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>00:00:00</t>
+          <t>00:39:40</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
@@ -4146,17 +4150,17 @@
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>5</t>
         </is>
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>5</t>
         </is>
       </c>
       <c r="K55" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="L55" t="inlineStr">
@@ -4171,38 +4175,38 @@
         </is>
       </c>
       <c r="O55" s="2" t="n">
-        <v>0.02722222222222222</v>
+        <v>0.0275462962962963</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>12/05/2022</t>
+          <t>03/06/2022</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>בילגורי</t>
+          <t>בועז</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>בועז</t>
+          <t>בילגורי</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>מרוץ הלילה השני של מודיעין</t>
+          <t>מרוץ גני תקווה ה-3</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>367</t>
+          <t>546</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>00:19:41</t>
+          <t>00:39:12</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
@@ -4212,22 +4216,22 @@
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>5000</t>
+          <t>10 ק"מ</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>15</t>
         </is>
       </c>
       <c r="J56" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>15</t>
         </is>
       </c>
       <c r="K56" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="L56" t="inlineStr">
@@ -4238,88 +4242,88 @@
       <c r="M56" t="inlineStr"/>
       <c r="N56" t="inlineStr">
         <is>
-          <t>5K</t>
+          <t>10K</t>
         </is>
       </c>
       <c r="O56" s="2" t="n">
-        <v>0.01366898148148148</v>
+        <v>0.02722222222222222</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>01/04/2022</t>
+          <t>12/05/2022</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>בועז</t>
+          <t>בילגורי</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>בילגורי</t>
+          <t>בועז</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>מרוץ לוד 2022</t>
+          <t>מרוץ הלילה השני של מודיעין</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>278</t>
+          <t>367</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>00:39:03</t>
+          <t>00:19:41</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>00:39:03</t>
+          <t>00:00:00</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>10 ק"מ</t>
+          <t>5000</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>10</t>
         </is>
       </c>
       <c r="K57" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="L57" t="inlineStr">
         <is>
-          <t>40-49 M</t>
+          <t>ותיקים 40-49</t>
         </is>
       </c>
       <c r="M57" t="inlineStr"/>
       <c r="N57" t="inlineStr">
         <is>
-          <t>10K</t>
+          <t>5K</t>
         </is>
       </c>
       <c r="O57" s="2" t="n">
-        <v>0.02711805555555555</v>
+        <v>0.01366898148148148</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>25/02/2022</t>
+          <t>01/04/2022</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -4334,59 +4338,63 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>מרתון סמסונג תל אביב 2022</t>
-        </is>
-      </c>
-      <c r="E58" t="inlineStr"/>
+          <t>מרוץ לוד 2022</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>278</t>
+        </is>
+      </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>01:33:51</t>
+          <t>00:39:03</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>00:00:00</t>
+          <t>00:39:03</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>21097</t>
+          <t>10 ק"מ</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>397</t>
+          <t>15</t>
         </is>
       </c>
       <c r="J58" t="inlineStr">
         <is>
-          <t>377</t>
+          <t>14</t>
         </is>
       </c>
       <c r="K58" t="inlineStr">
         <is>
-          <t>63</t>
+          <t>2</t>
         </is>
       </c>
       <c r="L58" t="inlineStr">
         <is>
-          <t>גברים 44-40 21K</t>
+          <t>40-49 M</t>
         </is>
       </c>
       <c r="M58" t="inlineStr"/>
       <c r="N58" t="inlineStr">
         <is>
-          <t>21K</t>
+          <t>10K</t>
         </is>
       </c>
       <c r="O58" s="2" t="n">
-        <v>0.06517361111111111</v>
+        <v>0.02711805555555555</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>10/11/2021</t>
+          <t>25/02/2022</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -4401,13 +4409,13 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>מרוץ הלילה של תל אביב</t>
+          <t>מרתון סמסונג תל אביב 2022</t>
         </is>
       </c>
       <c r="E59" t="inlineStr"/>
       <c r="F59" t="inlineStr">
         <is>
-          <t>01:00:38</t>
+          <t>01:33:51</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
@@ -4417,43 +4425,43 @@
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>10 ק"מ</t>
+          <t>21097</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>4516</t>
+          <t>397</t>
         </is>
       </c>
       <c r="J59" t="inlineStr">
         <is>
-          <t>3661</t>
+          <t>377</t>
         </is>
       </c>
       <c r="K59" t="inlineStr">
         <is>
-          <t>1128</t>
+          <t>63</t>
         </is>
       </c>
       <c r="L59" t="inlineStr">
         <is>
-          <t>גברים 40-49</t>
+          <t>גברים 44-40 21K</t>
         </is>
       </c>
       <c r="M59" t="inlineStr"/>
       <c r="N59" t="inlineStr">
         <is>
-          <t>10K</t>
+          <t>21K</t>
         </is>
       </c>
       <c r="O59" s="2" t="n">
-        <v>0.04210648148148148</v>
+        <v>0.06517361111111111</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>07/10/2021</t>
+          <t>10/11/2021</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -4468,22 +4476,18 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>מרוץ הלילה של רחובות</t>
-        </is>
-      </c>
-      <c r="E60" t="inlineStr">
-        <is>
-          <t>135</t>
-        </is>
-      </c>
+          <t>מרוץ הלילה של תל אביב</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr"/>
       <c r="F60" t="inlineStr">
         <is>
-          <t>00:43:55</t>
+          <t>01:00:38</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>00:43:51</t>
+          <t>00:00:00</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
@@ -4493,22 +4497,22 @@
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>4516</t>
         </is>
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>3661</t>
         </is>
       </c>
       <c r="K60" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>1128</t>
         </is>
       </c>
       <c r="L60" t="inlineStr">
         <is>
-          <t>40-49 M</t>
+          <t>גברים 40-49</t>
         </is>
       </c>
       <c r="M60" t="inlineStr"/>
@@ -4518,13 +4522,13 @@
         </is>
       </c>
       <c r="O60" s="2" t="n">
-        <v>0.03045138888888889</v>
+        <v>0.04210648148148148</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>19/02/2021</t>
+          <t>07/10/2021</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -4539,39 +4543,63 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>מרתון תל אביב 2021</t>
-        </is>
-      </c>
-      <c r="E61" t="inlineStr"/>
+          <t>מרוץ הלילה של רחובות</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>135</t>
+        </is>
+      </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>01:43:37</t>
+          <t>00:43:55</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>00:00:00</t>
-        </is>
-      </c>
-      <c r="H61" t="inlineStr"/>
+          <t>00:43:51</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>10 ק"מ</t>
+        </is>
+      </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>121</t>
-        </is>
-      </c>
-      <c r="J61" t="inlineStr"/>
-      <c r="K61" t="inlineStr"/>
-      <c r="L61" t="inlineStr"/>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="L61" t="inlineStr">
+        <is>
+          <t>40-49 M</t>
+        </is>
+      </c>
       <c r="M61" t="inlineStr"/>
-      <c r="N61" t="inlineStr"/>
+      <c r="N61" t="inlineStr">
+        <is>
+          <t>10K</t>
+        </is>
+      </c>
       <c r="O61" s="2" t="n">
-        <v>0.07195601851851852</v>
+        <v>0.03045138888888889</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>30/10/2019</t>
+          <t>19/02/2021</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -4586,52 +4614,99 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>מרוץ הלילה של ת"א 2019</t>
+          <t>מרתון תל אביב 2021</t>
         </is>
       </c>
       <c r="E62" t="inlineStr"/>
       <c r="F62" t="inlineStr">
         <is>
+          <t>01:43:37</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>00:00:00</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr"/>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>121</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr"/>
+      <c r="K62" t="inlineStr"/>
+      <c r="L62" t="inlineStr"/>
+      <c r="M62" t="inlineStr"/>
+      <c r="N62" t="inlineStr"/>
+      <c r="O62" s="2" t="n">
+        <v>0.07195601851851852</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>30/10/2019</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>בועז</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>בילגורי</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>מרוץ הלילה של ת"א 2019</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr"/>
+      <c r="F63" t="inlineStr">
+        <is>
           <t>00:58:40</t>
         </is>
       </c>
-      <c r="G62" t="inlineStr">
+      <c r="G63" t="inlineStr">
         <is>
           <t>00:00:00</t>
         </is>
       </c>
-      <c r="H62" t="inlineStr">
+      <c r="H63" t="inlineStr">
         <is>
           <t>10 ק"מ</t>
         </is>
       </c>
-      <c r="I62" t="inlineStr">
+      <c r="I63" t="inlineStr">
         <is>
           <t>4667</t>
         </is>
       </c>
-      <c r="J62" t="inlineStr">
+      <c r="J63" t="inlineStr">
         <is>
           <t>3974</t>
         </is>
       </c>
-      <c r="K62" t="inlineStr">
+      <c r="K63" t="inlineStr">
         <is>
           <t>2134</t>
         </is>
       </c>
-      <c r="L62" t="inlineStr">
+      <c r="L63" t="inlineStr">
         <is>
           <t>גברים 20-39</t>
         </is>
       </c>
-      <c r="M62" t="inlineStr"/>
-      <c r="N62" t="inlineStr">
+      <c r="M63" t="inlineStr"/>
+      <c r="N63" t="inlineStr">
         <is>
           <t>10K</t>
         </is>
       </c>
-      <c r="O62" s="2" t="n">
+      <c r="O63" s="2" t="n">
         <v>0.04074074074074074</v>
       </c>
     </row>

</xml_diff>